<commit_message>
commit before pilot_23: fix boat instead of sailbaot for concept folder name
</commit_message>
<xml_diff>
--- a/psychopy_exp_files/sequences/localizer_conditions_things-meg_mixed_5cat_00.xlsx
+++ b/psychopy_exp_files/sequences/localizer_conditions_things-meg_mixed_5cat_00.xlsx
@@ -728,7 +728,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -742,12 +742,12 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>boat\boat_12.png</t>
+          <t>sailboat\sailboat_12.png</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -864,12 +864,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>boat\boat_11.png</t>
+          <t>sailboat\sailboat_11.png</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1243,7 +1243,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1598,7 +1598,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G19" t="n">
@@ -1612,12 +1612,12 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>boat\boat_05.png</t>
+          <t>sailboat\sailboat_05.png</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1781,7 +1781,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G22" t="n">
@@ -1795,12 +1795,12 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>boat\boat_10.png</t>
+          <t>sailboat\sailboat_10.png</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -1903,7 +1903,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G24" t="n">
@@ -1917,12 +1917,12 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>boat\boat_03.png</t>
+          <t>sailboat\sailboat_03.png</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -4070,7 +4070,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G59" t="n">
@@ -4084,12 +4084,12 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>boat\boat_01.png</t>
+          <t>sailboat\sailboat_01.png</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
@@ -5012,7 +5012,7 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
@@ -5306,7 +5306,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G79" t="n">
@@ -5320,12 +5320,12 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>boat\boat_08.png</t>
+          <t>sailboat\sailboat_08.png</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
@@ -5985,7 +5985,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G90" t="n">
@@ -5999,12 +5999,12 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>boat\boat_04.png</t>
+          <t>sailboat\sailboat_04.png</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
@@ -6420,7 +6420,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G97" t="n">
@@ -6434,12 +6434,12 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>boat\boat_13.png</t>
+          <t>sailboat\sailboat_13.png</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L97" t="inlineStr">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G101" t="n">
@@ -6678,12 +6678,12 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>boat\boat_06.png</t>
+          <t>sailboat\sailboat_06.png</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
@@ -7343,7 +7343,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G112" t="n">
@@ -7357,12 +7357,12 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>boat\boat_02.png</t>
+          <t>sailboat\sailboat_02.png</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
@@ -7587,7 +7587,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G116" t="n">
@@ -7601,12 +7601,12 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>boat\boat_09.png</t>
+          <t>sailboat\sailboat_09.png</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
@@ -8022,7 +8022,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G123" t="n">
@@ -8036,12 +8036,12 @@
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>boat\boat_08.png</t>
+          <t>sailboat\sailboat_08.png</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
@@ -9136,7 +9136,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G141" t="n">
@@ -9150,12 +9150,12 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>boat\boat_05.png</t>
+          <t>sailboat\sailboat_05.png</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L141" t="inlineStr">
@@ -9693,7 +9693,7 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G150" t="n">
@@ -9707,12 +9707,12 @@
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>boat\boat_07.png</t>
+          <t>sailboat\sailboat_07.png</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L150" t="inlineStr">
@@ -10128,7 +10128,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G157" t="n">
@@ -10142,12 +10142,12 @@
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>boat\boat_01.png</t>
+          <t>sailboat\sailboat_01.png</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L157" t="inlineStr">
@@ -10433,7 +10433,7 @@
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G162" t="n">
@@ -10447,12 +10447,12 @@
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>boat\boat_13.png</t>
+          <t>sailboat\sailboat_13.png</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L162" t="inlineStr">
@@ -11001,7 +11001,7 @@
       </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L171" t="inlineStr">
@@ -11425,7 +11425,7 @@
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G178" t="n">
@@ -11439,12 +11439,12 @@
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>boat\boat_03.png</t>
+          <t>sailboat\sailboat_03.png</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L178" t="inlineStr">
@@ -11547,7 +11547,7 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G180" t="n">
@@ -11561,12 +11561,12 @@
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>boat\boat_07.png</t>
+          <t>sailboat\sailboat_07.png</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L180" t="inlineStr">
@@ -12287,7 +12287,7 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G192" t="n">
@@ -12301,12 +12301,12 @@
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>boat\boat_12.png</t>
+          <t>sailboat\sailboat_12.png</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L192" t="inlineStr">
@@ -14011,7 +14011,7 @@
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G220" t="n">
@@ -14025,7 +14025,7 @@
       </c>
       <c r="J220" t="inlineStr">
         <is>
-          <t>boat\boat_06.png</t>
+          <t>sailboat\sailboat_06.png</t>
         </is>
       </c>
       <c r="K220" t="inlineStr">
@@ -14454,7 +14454,7 @@
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G227" t="n">
@@ -14468,12 +14468,12 @@
       </c>
       <c r="J227" t="inlineStr">
         <is>
-          <t>boat\boat_11.png</t>
+          <t>sailboat\sailboat_11.png</t>
         </is>
       </c>
       <c r="K227" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L227" t="inlineStr">
@@ -14820,7 +14820,7 @@
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G233" t="n">
@@ -14834,12 +14834,12 @@
       </c>
       <c r="J233" t="inlineStr">
         <is>
-          <t>boat\boat_09.png</t>
+          <t>sailboat\sailboat_09.png</t>
         </is>
       </c>
       <c r="K233" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L233" t="inlineStr">
@@ -15682,7 +15682,7 @@
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G247" t="n">
@@ -15696,12 +15696,12 @@
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>boat\boat_10.png</t>
+          <t>sailboat\sailboat_10.png</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L247" t="inlineStr">
@@ -15804,7 +15804,7 @@
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G249" t="n">
@@ -15818,12 +15818,12 @@
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>boat\boat_04.png</t>
+          <t>sailboat\sailboat_04.png</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L249" t="inlineStr">
@@ -16056,7 +16056,7 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G253" t="n">
@@ -16070,12 +16070,12 @@
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>boat\boat_02.png</t>
+          <t>sailboat\sailboat_02.png</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L253" t="inlineStr">
@@ -16319,7 +16319,7 @@
       </c>
       <c r="K257" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L257" t="inlineStr">
@@ -17353,7 +17353,7 @@
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G274" t="n">
@@ -17367,12 +17367,12 @@
       </c>
       <c r="J274" t="inlineStr">
         <is>
-          <t>boat\boat_01.png</t>
+          <t>sailboat\sailboat_01.png</t>
         </is>
       </c>
       <c r="K274" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L274" t="inlineStr">
@@ -18780,7 +18780,7 @@
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G297" t="n">
@@ -18794,12 +18794,12 @@
       </c>
       <c r="J297" t="inlineStr">
         <is>
-          <t>boat\boat_12.png</t>
+          <t>sailboat\sailboat_12.png</t>
         </is>
       </c>
       <c r="K297" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L297" t="inlineStr">
@@ -18902,7 +18902,7 @@
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G299" t="n">
@@ -18916,12 +18916,12 @@
       </c>
       <c r="J299" t="inlineStr">
         <is>
-          <t>boat\boat_10.png</t>
+          <t>sailboat\sailboat_10.png</t>
         </is>
       </c>
       <c r="K299" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L299" t="inlineStr">
@@ -19024,7 +19024,7 @@
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G301" t="n">
@@ -19038,12 +19038,12 @@
       </c>
       <c r="J301" t="inlineStr">
         <is>
-          <t>boat\boat_09.png</t>
+          <t>sailboat\sailboat_09.png</t>
         </is>
       </c>
       <c r="K301" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L301" t="inlineStr">
@@ -19146,7 +19146,7 @@
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G303" t="n">
@@ -19160,12 +19160,12 @@
       </c>
       <c r="J303" t="inlineStr">
         <is>
-          <t>boat\boat_04.png</t>
+          <t>sailboat\sailboat_04.png</t>
         </is>
       </c>
       <c r="K303" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L303" t="inlineStr">
@@ -20321,7 +20321,7 @@
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G322" t="n">
@@ -20335,12 +20335,12 @@
       </c>
       <c r="J322" t="inlineStr">
         <is>
-          <t>boat\boat_07.png</t>
+          <t>sailboat\sailboat_07.png</t>
         </is>
       </c>
       <c r="K322" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L322" t="inlineStr">
@@ -20504,7 +20504,7 @@
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G325" t="n">
@@ -20518,12 +20518,12 @@
       </c>
       <c r="J325" t="inlineStr">
         <is>
-          <t>boat\boat_05.png</t>
+          <t>sailboat\sailboat_05.png</t>
         </is>
       </c>
       <c r="K325" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L325" t="inlineStr">
@@ -20748,7 +20748,7 @@
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G329" t="n">
@@ -20762,7 +20762,7 @@
       </c>
       <c r="J329" t="inlineStr">
         <is>
-          <t>boat\boat_03.png</t>
+          <t>sailboat\sailboat_03.png</t>
         </is>
       </c>
       <c r="K329" t="inlineStr">
@@ -21557,7 +21557,7 @@
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G342" t="n">
@@ -21571,12 +21571,12 @@
       </c>
       <c r="J342" t="inlineStr">
         <is>
-          <t>boat\boat_11.png</t>
+          <t>sailboat\sailboat_11.png</t>
         </is>
       </c>
       <c r="K342" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L342" t="inlineStr">
@@ -22236,7 +22236,7 @@
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G353" t="n">
@@ -22250,12 +22250,12 @@
       </c>
       <c r="J353" t="inlineStr">
         <is>
-          <t>boat\boat_06.png</t>
+          <t>sailboat\sailboat_06.png</t>
         </is>
       </c>
       <c r="K353" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L353" t="inlineStr">
@@ -22541,7 +22541,7 @@
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G358" t="n">
@@ -22555,7 +22555,7 @@
       </c>
       <c r="J358" t="inlineStr">
         <is>
-          <t>boat\boat_08.png</t>
+          <t>sailboat\sailboat_08.png</t>
         </is>
       </c>
       <c r="K358" t="inlineStr">
@@ -24204,7 +24204,7 @@
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G385" t="n">
@@ -24218,12 +24218,12 @@
       </c>
       <c r="J385" t="inlineStr">
         <is>
-          <t>boat\boat_02.png</t>
+          <t>sailboat\sailboat_02.png</t>
         </is>
       </c>
       <c r="K385" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L385" t="inlineStr">
@@ -24517,7 +24517,7 @@
       </c>
       <c r="F390" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G390" t="n">
@@ -24531,12 +24531,12 @@
       </c>
       <c r="J390" t="inlineStr">
         <is>
-          <t>boat\boat_10.png</t>
+          <t>sailboat\sailboat_10.png</t>
         </is>
       </c>
       <c r="K390" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L390" t="inlineStr">
@@ -25196,7 +25196,7 @@
       </c>
       <c r="F401" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G401" t="n">
@@ -25210,12 +25210,12 @@
       </c>
       <c r="J401" t="inlineStr">
         <is>
-          <t>boat\boat_13.png</t>
+          <t>sailboat\sailboat_13.png</t>
         </is>
       </c>
       <c r="K401" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L401" t="inlineStr">
@@ -26310,7 +26310,7 @@
       </c>
       <c r="F419" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G419" t="n">
@@ -26324,12 +26324,12 @@
       </c>
       <c r="J419" t="inlineStr">
         <is>
-          <t>boat\boat_03.png</t>
+          <t>sailboat\sailboat_03.png</t>
         </is>
       </c>
       <c r="K419" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L419" t="inlineStr">
@@ -26554,7 +26554,7 @@
       </c>
       <c r="F423" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G423" t="n">
@@ -26568,12 +26568,12 @@
       </c>
       <c r="J423" t="inlineStr">
         <is>
-          <t>boat\boat_08.png</t>
+          <t>sailboat\sailboat_08.png</t>
         </is>
       </c>
       <c r="K423" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L423" t="inlineStr">
@@ -27286,7 +27286,7 @@
       </c>
       <c r="F435" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G435" t="n">
@@ -27300,7 +27300,7 @@
       </c>
       <c r="J435" t="inlineStr">
         <is>
-          <t>boat\boat_09.png</t>
+          <t>sailboat\sailboat_09.png</t>
         </is>
       </c>
       <c r="K435" t="inlineStr">
@@ -27740,7 +27740,7 @@
       </c>
       <c r="K442" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L442" t="inlineStr">
@@ -27851,7 +27851,7 @@
       </c>
       <c r="F444" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G444" t="n">
@@ -27865,12 +27865,12 @@
       </c>
       <c r="J444" t="inlineStr">
         <is>
-          <t>boat\boat_01.png</t>
+          <t>sailboat\sailboat_01.png</t>
         </is>
       </c>
       <c r="K444" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L444" t="inlineStr">
@@ -28278,7 +28278,7 @@
       </c>
       <c r="F451" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G451" t="n">
@@ -28292,12 +28292,12 @@
       </c>
       <c r="J451" t="inlineStr">
         <is>
-          <t>boat\boat_02.png</t>
+          <t>sailboat\sailboat_02.png</t>
         </is>
       </c>
       <c r="K451" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L451" t="inlineStr">
@@ -28591,7 +28591,7 @@
       </c>
       <c r="F456" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G456" t="n">
@@ -28605,12 +28605,12 @@
       </c>
       <c r="J456" t="inlineStr">
         <is>
-          <t>boat\boat_04.png</t>
+          <t>sailboat\sailboat_04.png</t>
         </is>
       </c>
       <c r="K456" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L456" t="inlineStr">
@@ -29018,7 +29018,7 @@
       </c>
       <c r="F463" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G463" t="n">
@@ -29032,12 +29032,12 @@
       </c>
       <c r="J463" t="inlineStr">
         <is>
-          <t>boat\boat_06.png</t>
+          <t>sailboat\sailboat_06.png</t>
         </is>
       </c>
       <c r="K463" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L463" t="inlineStr">
@@ -29819,7 +29819,7 @@
       </c>
       <c r="F476" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G476" t="n">
@@ -29833,12 +29833,12 @@
       </c>
       <c r="J476" t="inlineStr">
         <is>
-          <t>boat\boat_11.png</t>
+          <t>sailboat\sailboat_11.png</t>
         </is>
       </c>
       <c r="K476" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L476" t="inlineStr">
@@ -30429,7 +30429,7 @@
       </c>
       <c r="F486" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G486" t="n">
@@ -30443,12 +30443,12 @@
       </c>
       <c r="J486" t="inlineStr">
         <is>
-          <t>boat\boat_12.png</t>
+          <t>sailboat\sailboat_12.png</t>
         </is>
       </c>
       <c r="K486" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L486" t="inlineStr">
@@ -30681,7 +30681,7 @@
       </c>
       <c r="F490" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G490" t="n">
@@ -30695,7 +30695,7 @@
       </c>
       <c r="J490" t="inlineStr">
         <is>
-          <t>boat\boat_05.png</t>
+          <t>sailboat\sailboat_05.png</t>
         </is>
       </c>
       <c r="K490" t="inlineStr">
@@ -31482,7 +31482,7 @@
       </c>
       <c r="F503" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G503" t="n">
@@ -31496,12 +31496,12 @@
       </c>
       <c r="J503" t="inlineStr">
         <is>
-          <t>boat\boat_03.png</t>
+          <t>sailboat\sailboat_03.png</t>
         </is>
       </c>
       <c r="K503" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L503" t="inlineStr">
@@ -31909,7 +31909,7 @@
       </c>
       <c r="F510" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G510" t="n">
@@ -31923,7 +31923,7 @@
       </c>
       <c r="J510" t="inlineStr">
         <is>
-          <t>boat\boat_07.png</t>
+          <t>sailboat\sailboat_07.png</t>
         </is>
       </c>
       <c r="K510" t="inlineStr">
@@ -32535,7 +32535,7 @@
       </c>
       <c r="F520" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G520" t="n">
@@ -32549,12 +32549,12 @@
       </c>
       <c r="J520" t="inlineStr">
         <is>
-          <t>boat\boat_01.png</t>
+          <t>sailboat\sailboat_01.png</t>
         </is>
       </c>
       <c r="K520" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L520" t="inlineStr">
@@ -33206,7 +33206,7 @@
       </c>
       <c r="F531" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G531" t="n">
@@ -33220,12 +33220,12 @@
       </c>
       <c r="J531" t="inlineStr">
         <is>
-          <t>boat\boat_13.png</t>
+          <t>sailboat\sailboat_13.png</t>
         </is>
       </c>
       <c r="K531" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L531" t="inlineStr">
@@ -33824,7 +33824,7 @@
       </c>
       <c r="F541" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G541" t="n">
@@ -33838,12 +33838,12 @@
       </c>
       <c r="J541" t="inlineStr">
         <is>
-          <t>boat\boat_12.png</t>
+          <t>sailboat\sailboat_12.png</t>
         </is>
       </c>
       <c r="K541" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L541" t="inlineStr">
@@ -35182,7 +35182,7 @@
       </c>
       <c r="F563" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G563" t="n">
@@ -35196,12 +35196,12 @@
       </c>
       <c r="J563" t="inlineStr">
         <is>
-          <t>boat\boat_05.png</t>
+          <t>sailboat\sailboat_05.png</t>
         </is>
       </c>
       <c r="K563" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L563" t="inlineStr">
@@ -36349,7 +36349,7 @@
       </c>
       <c r="F582" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G582" t="n">
@@ -36363,12 +36363,12 @@
       </c>
       <c r="J582" t="inlineStr">
         <is>
-          <t>boat\boat_08.png</t>
+          <t>sailboat\sailboat_08.png</t>
         </is>
       </c>
       <c r="K582" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L582" t="inlineStr">
@@ -36471,7 +36471,7 @@
       </c>
       <c r="F584" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G584" t="n">
@@ -36485,12 +36485,12 @@
       </c>
       <c r="J584" t="inlineStr">
         <is>
-          <t>boat\boat_13.png</t>
+          <t>sailboat\sailboat_13.png</t>
         </is>
       </c>
       <c r="K584" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L584" t="inlineStr">
@@ -36776,7 +36776,7 @@
       </c>
       <c r="F589" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G589" t="n">
@@ -36790,12 +36790,12 @@
       </c>
       <c r="J589" t="inlineStr">
         <is>
-          <t>boat\boat_04.png</t>
+          <t>sailboat\sailboat_04.png</t>
         </is>
       </c>
       <c r="K589" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L589" t="inlineStr">
@@ -37402,7 +37402,7 @@
       </c>
       <c r="F599" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G599" t="n">
@@ -37416,12 +37416,12 @@
       </c>
       <c r="J599" t="inlineStr">
         <is>
-          <t>boat\boat_09.png</t>
+          <t>sailboat\sailboat_09.png</t>
         </is>
       </c>
       <c r="K599" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L599" t="inlineStr">
@@ -37585,7 +37585,7 @@
       </c>
       <c r="F602" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G602" t="n">
@@ -37599,12 +37599,12 @@
       </c>
       <c r="J602" t="inlineStr">
         <is>
-          <t>boat\boat_07.png</t>
+          <t>sailboat\sailboat_07.png</t>
         </is>
       </c>
       <c r="K602" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L602" t="inlineStr">
@@ -38214,7 +38214,7 @@
       </c>
       <c r="K612" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L612" t="inlineStr">
@@ -38882,7 +38882,7 @@
       </c>
       <c r="F623" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G623" t="n">
@@ -38896,12 +38896,12 @@
       </c>
       <c r="J623" t="inlineStr">
         <is>
-          <t>boat\boat_06.png</t>
+          <t>sailboat\sailboat_06.png</t>
         </is>
       </c>
       <c r="K623" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L623" t="inlineStr">
@@ -39004,7 +39004,7 @@
       </c>
       <c r="F625" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G625" t="n">
@@ -39018,12 +39018,12 @@
       </c>
       <c r="J625" t="inlineStr">
         <is>
-          <t>boat\boat_10.png</t>
+          <t>sailboat\sailboat_10.png</t>
         </is>
       </c>
       <c r="K625" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L625" t="inlineStr">
@@ -39126,7 +39126,7 @@
       </c>
       <c r="F627" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G627" t="n">
@@ -39140,12 +39140,12 @@
       </c>
       <c r="J627" t="inlineStr">
         <is>
-          <t>boat\boat_11.png</t>
+          <t>sailboat\sailboat_11.png</t>
         </is>
       </c>
       <c r="K627" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L627" t="inlineStr">
@@ -39431,7 +39431,7 @@
       </c>
       <c r="F632" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="G632" t="n">
@@ -39445,12 +39445,12 @@
       </c>
       <c r="J632" t="inlineStr">
         <is>
-          <t>boat\boat_02.png</t>
+          <t>sailboat\sailboat_02.png</t>
         </is>
       </c>
       <c r="K632" t="inlineStr">
         <is>
-          <t>boat</t>
+          <t>sailboat</t>
         </is>
       </c>
       <c r="L632" t="inlineStr">

</xml_diff>